<commit_message>
Planilha: coluna N vira Curva da Assessoria, nova coluna O Curva ABC análise do Claude
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos enviados/PLANEJADOR DE FBA.xlsx
+++ b/arquivos enviados/PLANEJADOR DE FBA.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:N39"/>
+  <dimension ref="A2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23.5703125" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,8 @@
     <col width="30.5703125" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="15.85546875" customWidth="1" min="12" max="12"/>
     <col width="25.5703125" bestFit="1" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -542,6 +543,26 @@
           <t>CURVA</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>ASIN</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Curva da Assessoria</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Curva ABC análise do Claude</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -579,17 +600,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>ASIN</t>
+          <t>B0GW9K8BFW</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>sku</t>
+          <t>COLHER-MAD-30-1_FBA</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Curva </t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -629,15 +655,20 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>B0GW9K8BFW</t>
+          <t>B0GV5M89QB</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>COLHER-MAD-30-1_FBA</t>
+          <t>COLHER-MAD-38-1_FBA</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -679,17 +710,22 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>B0GV5M89QB</t>
+          <t>B0GW1B2W11</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>COLHER-MAD-38-1_FBA</t>
+          <t>ROL_MAS_M_FBA</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -729,15 +765,20 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>B0GW1B2W11</t>
+          <t>B0GW16ZJ3Y</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>ROL_MAS_M_FBA</t>
+          <t>ROL_MAS_P_FBA</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -779,17 +820,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>B0GW16ZJ3Y</t>
+          <t>B0GW9KS8PV</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ROL_MAS_P_FBA</t>
+          <t>COLHER-MAD-26-1_FBA</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -829,15 +875,20 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>B0GW9KS8PV</t>
+          <t>B0H1MXYGWT</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>COLHER-MAD-26-1_FBA</t>
+          <t>COLHER-MAD-26-5_FBA</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -879,15 +930,20 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>B0H1MXYGWT</t>
+          <t>B0H1N3NWC6</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>COLHER-MAD-26-5_FBA</t>
+          <t>COLHER-MAD-30-5_FBA</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -929,17 +985,22 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>B0H1N3NWC6</t>
+          <t>B0H1N71MTD</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>COLHER-MAD-30-5_FBA</t>
+          <t>COLHER-MAD-38-5_FBA</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -979,17 +1040,22 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>B0H1N71MTD</t>
+          <t>B0H1MWJ85Q</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>COLHER-MAD-38-5_FBA</t>
+          <t>KIT_ROL_FBA</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1029,15 +1095,20 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>B0H1MWJ85Q</t>
+          <t>B0GXGWGTYT</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>KIT_ROL_FBA</t>
+          <t>MESA_DOB_FBA</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1079,17 +1150,22 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>B0GXGWGTYT</t>
+          <t>B0GXGMPLTS</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>MESA_DOB_FBA</t>
+          <t>PILAO_M_FBA</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1205,22 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>B0GXGMPLTS</t>
+          <t>B0GZCTP3V2</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>PILAO_M_FBA</t>
+          <t>MEI-TERM-12_FBA</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1179,17 +1260,22 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>B0GZCTP3V2</t>
+          <t>B0GXGZHMMN</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>MEI-TERM-12_FBA</t>
+          <t>PILAO_G_FBA</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1229,15 +1315,20 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>B0GXGZHMMN</t>
+          <t>B0GXGNPF5N</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>PILAO_G_FBA</t>
+          <t>PILAO_P_FBA</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1279,15 +1370,20 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>B0GXGNPF5N</t>
+          <t>B0GXGPH3Z6</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>PILAO_P_FBA</t>
+          <t>PRATO_M_1_FBA</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1329,15 +1425,20 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>B0GXGPH3Z6</t>
+          <t>B0H1N9FKZY</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>PRATO_M_1_FBA</t>
+          <t>TAB_COR_G_2_FBA</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1379,17 +1480,22 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>B0H1N9FKZY</t>
+          <t>B0GXGTRJWC</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>TAB_COR_G_2_FBA</t>
+          <t>TAB_COR_M_FBA</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1429,15 +1535,15 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>B0GXGTRJWC</t>
+          <t>B0H1PGND8W</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>TAB_COR_M_FBA</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
+          <t>KIT_TAB_COR_1_FBA</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1479,12 +1585,17 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>B0H1PGND8W</t>
+          <t>B0H1STZBPJ</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>KIT_TAB_COR_1_FBA</t>
+          <t>PILAO_G_2_FBA</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1524,12 +1635,17 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>B0H1STZBPJ</t>
+          <t>B0H1SZBJRR</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>PILAO_G_2_FBA</t>
+          <t>PILAO_M_2_FBA</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1569,12 +1685,17 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>B0H1SZBJRR</t>
+          <t>B0H2WY3HG8</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>PILAO_M_2_FBA</t>
+          <t>PILAO_P_2_FBA</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1614,12 +1735,17 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>B0H2WY3HG8</t>
+          <t>B0GXGP9CMF</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>PILAO_P_2_FBA</t>
+          <t>PRATO_G_1_FBA</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1785,17 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>B0GXGP9CMF</t>
+          <t>B0GXH1JX31</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>PRATO_G_1_FBA</t>
+          <t>PRATO_P_1_FBA</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1704,12 +1835,17 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>B0GXH1JX31</t>
+          <t>B0GXGYTZJB</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>PRATO_P_1_FBA</t>
+          <t>TAB_COR_G_FBA</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1749,12 +1885,17 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>B0GXGYTZJB</t>
+          <t>B0H1P9YQX7</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>TAB_COR_G_FBA</t>
+          <t>TAB_COR_M_2_FBA</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1935,17 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>B0H1P9YQX7</t>
+          <t>B0H1P38Y8Y</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>TAB_COR_M_2_FBA</t>
+          <t>TAB_COR_P_2_FBA</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1839,12 +1985,17 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>B0H1P38Y8Y</t>
+          <t>B0GXGKJR1D</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>TAB_COR_P_2_FBA</t>
+          <t>TAB_COR_P_FBA</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1884,12 +2035,17 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>B0GXGKJR1D</t>
+          <t>B0GXXRDMS1</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>TAB_COR_P_FBA</t>
+          <t>TOA_BAN_DOU_FBA</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1929,12 +2085,17 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>B0GXXRDMS1</t>
+          <t>B0HHJZ4PHZ</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>TOA_BAN_DOU_FBA</t>
+          <t>TOA_BAN_ROS_2_FBA</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -1974,12 +2135,17 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>B0HHJZ4PHZ</t>
+          <t>B0HBFCCN6Y</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>TOA_BAN_ROS_2_FBA</t>
+          <t>TOA_COLORE_1_FBA</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -2019,27 +2185,21 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>B0HBFCCN6Y</t>
+          <t>B0HHJZF6HR</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>TOA_COLORE_1_FBA</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>B0HHJZF6HR</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
           <t>TOA_RUBI_2_FBA</t>
         </is>
       </c>
-    </row>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
     <row r="35"/>
     <row r="36"/>
     <row r="37"/>

</xml_diff>

<commit_message>
Envio3: planilha atualizada (inventário FBA, vendas 30d, curva ABC Claude)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos enviados/PLANEJADOR DE FBA.xlsx
+++ b/arquivos enviados/PLANEJADOR DE FBA.xlsx
@@ -582,7 +582,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>B0GXGMPLTS</t>
+          <t>B0GXGP9CMF</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
@@ -592,7 +592,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>0</v>
@@ -604,10 +604,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J3" s="1">
         <f>IFERROR(VLOOKUP(A3,L:N,3,0),"")</f>
@@ -637,14 +637,14 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>B0HHJZF6HR</t>
+          <t>B0GW16ZJ3Y</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
@@ -659,10 +659,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="J4" s="1">
         <f>IFERROR(VLOOKUP(A4,L:N,3,0),"")</f>
@@ -692,17 +692,17 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>B0GXGZHMMN</t>
+          <t>B0H1P38Y8Y</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>
@@ -714,10 +714,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J5" s="1">
         <f>IFERROR(VLOOKUP(A5,L:N,3,0),"")</f>
@@ -747,17 +747,17 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>B0GXGP9CMF</t>
+          <t>B0H1STZBPJ</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
@@ -769,7 +769,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I6" s="1" t="n">
         <v>0</v>
@@ -802,17 +802,17 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>B0H1P38Y8Y</t>
+          <t>B0GXGZHMMN</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0</v>
@@ -824,10 +824,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7" s="1">
         <f>IFERROR(VLOOKUP(A7,L:N,3,0),"")</f>
@@ -857,7 +857,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>B0H1STZBPJ</t>
+          <t>B0GXGYTZJB</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
@@ -912,14 +912,14 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>B0GXGYTZJB</t>
+          <t>B0HHJZ4PHZ</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>B0HHJZ4PHZ</t>
+          <t>B0HBFCCN6Y</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
@@ -1022,7 +1022,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>B0HBFCCN6Y</t>
+          <t>B0HHJZF6HR</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
@@ -1132,17 +1132,17 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>B0GW16ZJ3Y</t>
+          <t>B0GXXRDMS1</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
@@ -1157,7 +1157,7 @@
         <v>7</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J13" s="1">
         <f>IFERROR(VLOOKUP(A13,L:N,3,0),"")</f>
@@ -1180,24 +1180,24 @@
       </c>
       <c r="O13" s="1" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>B0GXXRDMS1</t>
+          <t>B0H1N9FKZY</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0</v>
@@ -1209,10 +1209,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="1">
         <f>IFERROR(VLOOKUP(A14,L:N,3,0),"")</f>
@@ -1242,7 +1242,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>B0H1N9FKZY</t>
+          <t>B0H1SZBJRR</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="1">
         <f>IFERROR(VLOOKUP(A15,L:N,3,0),"")</f>
@@ -1297,7 +1297,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>B0H1SZBJRR</t>
+          <t>B0H2WY3HG8</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
@@ -1352,7 +1352,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>B0H2WY3HG8</t>
+          <t>B0H1P9YQX7</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
@@ -1407,17 +1407,17 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>B0H1P9YQX7</t>
+          <t>B0H1MWJ85Q</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0</v>
@@ -1429,7 +1429,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I18" s="1" t="n">
         <v>0</v>
@@ -1462,7 +1462,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>B0H1MWJ85Q</t>
+          <t>B0GXGPH3Z6</t>
         </is>
       </c>
       <c r="B19" s="1" t="n">
@@ -1517,17 +1517,17 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>B0GXGPH3Z6</t>
+          <t>B0H1PGND8W</t>
         </is>
       </c>
       <c r="B20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="C20" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="D20" s="1" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>0</v>
@@ -1539,7 +1539,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>0</v>
@@ -1567,17 +1567,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>B0H1PGND8W</t>
+          <t>B0GXGMPLTS</t>
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>0</v>
@@ -1589,10 +1589,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I21" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" s="1">
         <f>IFERROR(VLOOKUP(A21,L:N,3,0),"")</f>
@@ -1717,14 +1717,14 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>B0GXGTRJWC</t>
+          <t>B0GW9K8BFW</t>
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>0</v>
@@ -1739,10 +1739,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J24" s="1">
         <f>IFERROR(VLOOKUP(A24,L:N,3,0),"")</f>
@@ -1767,32 +1767,32 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>B0H1N3NWC6</t>
+          <t>B0GXGTRJWC</t>
         </is>
       </c>
       <c r="B25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I25" s="1" t="n">
         <v>3</v>
-      </c>
-      <c r="C25" s="1" t="n">
-        <v>37</v>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="1" t="n">
-        <v>37</v>
-      </c>
-      <c r="I25" s="1" t="n">
-        <v>8</v>
       </c>
       <c r="J25" s="1">
         <f>IFERROR(VLOOKUP(A25,L:N,3,0),"")</f>
@@ -1817,14 +1817,14 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>B0GW9K8BFW</t>
+          <t>B0H1N3NWC6</t>
         </is>
       </c>
       <c r="B26" s="1" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>0</v>
@@ -1839,10 +1839,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="1" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J26" s="1">
         <f>IFERROR(VLOOKUP(A26,L:N,3,0),"")</f>
@@ -1921,10 +1921,10 @@
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C28" s="1" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D28" s="1" t="n">
         <v>0</v>
@@ -2021,10 +2021,10 @@
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D30" s="1" t="n">
         <v>0</v>
@@ -2039,10 +2039,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="1" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="J30" s="1">
         <f>IFERROR(VLOOKUP(A30,L:N,3,0),"")</f>
@@ -2071,10 +2071,10 @@
         </is>
       </c>
       <c r="B31" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D31" s="1" t="n">
         <v>0</v>
@@ -2089,7 +2089,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="1" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I31" s="1" t="n">
         <v>0</v>
@@ -2142,7 +2142,7 @@
         <v>91</v>
       </c>
       <c r="I32" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J32" s="1">
         <f>IFERROR(VLOOKUP(A32,L:N,3,0),"")</f>
@@ -2171,10 +2171,10 @@
         </is>
       </c>
       <c r="B33" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D33" s="1" t="n">
         <v>0</v>

</xml_diff>